<commit_message>
feat: update H3 downloads and workbench reliability
</commit_message>
<xml_diff>
--- a/jyd_plain_json_probe/apps/processor/frontend/new/project-script-template.xlsx
+++ b/jyd_plain_json_probe/apps/processor/frontend/new/project-script-template.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="脚本导入模板" sheetId="1" r:id="R0093838ac90a4c55"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="脚本导入模板" sheetId="1" r:id="Re70ee4e28eb8491c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -403,40 +403,20 @@
       <x:c r="B2" s="12" t="str">
         <x:v>请在这里填写第一条需要生成视频的完整脚本文案。</x:v>
       </x:c>
-      <x:c r="C2" s="22" t="str">
-        <x:v>干货类</x:v>
-      </x:c>
-      <x:c r="D2" s="20" t="str">
-        <x:v>1</x:v>
-      </x:c>
+      <x:c r="C2" s="22"/>
+      <x:c r="D2" s="20"/>
     </x:row>
     <x:row r="3" ht="32" customHeight="1">
-      <x:c r="A3" s="11" t="str">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="B3" s="12" t="str">
-        <x:v>请在这里填写第二条脚本文案，每一行对应一个视频任务。</x:v>
-      </x:c>
-      <x:c r="C3" s="22" t="str">
-        <x:v>鸡汤文</x:v>
-      </x:c>
-      <x:c r="D3" s="20" t="str">
-        <x:v>2</x:v>
-      </x:c>
+      <x:c r="A3" s="11"/>
+      <x:c r="B3" s="12"/>
+      <x:c r="C3" s="22"/>
+      <x:c r="D3" s="20"/>
     </x:row>
     <x:row r="4" ht="32" customHeight="1">
-      <x:c r="A4" s="13" t="str">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="B4" s="14" t="str">
-        <x:v>任务ID用于编号，必须唯一；脚本内容不能为空。</x:v>
-      </x:c>
-      <x:c r="C4" s="23" t="str">
-        <x:v>带人设介绍的干货类</x:v>
-      </x:c>
-      <x:c r="D4" s="21" t="str">
-        <x:v>3</x:v>
-      </x:c>
+      <x:c r="A4" s="13"/>
+      <x:c r="B4" s="14"/>
+      <x:c r="C4" s="23"/>
+      <x:c r="D4" s="21"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>